<commit_message>
Unificação dos vendedores SP, MG e blacklists em um unico xlsx. Ajuste na prioridade da comissão de simuladores com prejuizo
</commit_message>
<xml_diff>
--- a/comissoes_fixas.xlsx
+++ b/comissoes_fixas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\TI\ROBERT\PROJETO COMISSOES\Script\extrator_comissoes_relatorio_final\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{475694F0-4CA1-42D5-8220-A834D7AFE2A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C1AA691-34EE-4CA4-9824-128DCD224CDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>CLIENTE</t>
   </si>
@@ -76,6 +76,9 @@
   </si>
   <si>
     <t>STRATOS LTDA</t>
+  </si>
+  <si>
+    <t>FOSPAR S/A</t>
   </si>
 </sst>
 </file>
@@ -431,7 +434,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="39" bestFit="1" customWidth="1"/>
@@ -552,9 +555,17 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="2">
+        <v>5.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="2">
+      <c r="B16" s="2">
         <v>5.0000000000000001E-3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajuste nas tabelas de comissoes fixas e vendedores
</commit_message>
<xml_diff>
--- a/comissoes_fixas.xlsx
+++ b/comissoes_fixas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\TI\ROBERT\PROJETO COMISSOES\Script\extrator_comissoes_relatorio_final\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C1AA691-34EE-4CA4-9824-128DCD224CDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83471F48-94B8-449E-B7D4-02FACC8A147A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>CLIENTE</t>
   </si>
@@ -79,6 +79,12 @@
   </si>
   <si>
     <t>FOSPAR S/A</t>
+  </si>
+  <si>
+    <t>MARGEM</t>
+  </si>
+  <si>
+    <t>COMISSAO CONDICIONAL</t>
   </si>
 </sst>
 </file>
@@ -434,139 +440,237 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr defaultColWidth="15.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="39" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.7109375" customWidth="1"/>
+    <col min="2" max="2" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="2">
         <v>5.0000000000000001E-3</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C2" s="2">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="D2" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="2">
         <v>7.0000000000000001E-3</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C3" s="2">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="D3" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="2">
         <v>7.0000000000000001E-3</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C4" s="2">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="D4" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B5" s="2">
         <v>7.0000000000000001E-3</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C5" s="2">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="D5" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B6" s="2">
         <v>7.0000000000000001E-3</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C6" s="2">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="D6" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B7" s="2">
         <v>7.0000000000000001E-3</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C7" s="2">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="D7" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B8" s="2">
         <v>7.0000000000000001E-3</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C8" s="2">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="D8" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>9</v>
       </c>
       <c r="B9" s="2">
-        <v>5.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="C9" s="2">
+        <v>0.02</v>
+      </c>
+      <c r="D9" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B10" s="2">
-        <v>5.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="C10" s="2">
+        <v>0.02</v>
+      </c>
+      <c r="D10" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>11</v>
       </c>
       <c r="B11" s="2">
-        <v>5.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="C11" s="2">
+        <v>0.02</v>
+      </c>
+      <c r="D11" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>12</v>
       </c>
       <c r="B12" s="2">
-        <v>5.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="C12" s="2">
+        <v>0.02</v>
+      </c>
+      <c r="D12" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>13</v>
       </c>
       <c r="B13" s="2">
-        <v>5.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="C13" s="2">
+        <v>0.02</v>
+      </c>
+      <c r="D13" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B14" s="2">
-        <v>5.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="C14" s="2">
+        <v>0.02</v>
+      </c>
+      <c r="D14" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>16</v>
       </c>
       <c r="B15" s="2">
-        <v>5.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="C15" s="2">
+        <v>0.02</v>
+      </c>
+      <c r="D15" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B16" s="2">
-        <v>5.0000000000000001E-3</v>
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="C16" s="2">
+        <v>0.02</v>
+      </c>
+      <c r="D16" s="2">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Inserção do json no Banco de Dados, de maneira provisória
</commit_message>
<xml_diff>
--- a/comissoes_fixas.xlsx
+++ b/comissoes_fixas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\TI\ROBERT\PROJETO COMISSOES\Script\extrator_comissoes_relatorio_final\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83471F48-94B8-449E-B7D4-02FACC8A147A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{621A5635-3D45-4D42-ABA8-3A15A58851B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>CLIENTE</t>
   </si>
@@ -85,6 +85,12 @@
   </si>
   <si>
     <t>COMISSAO CONDICIONAL</t>
+  </si>
+  <si>
+    <t>ALCOA</t>
+  </si>
+  <si>
+    <t>CONSORCIO ALUMAR</t>
   </si>
 </sst>
 </file>
@@ -440,7 +446,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr defaultColWidth="15.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="39" bestFit="1" customWidth="1"/>
@@ -479,13 +485,13 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="B3" s="2">
-        <v>7.0000000000000001E-3</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="C3" s="2">
-        <v>7.0000000000000001E-3</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="D3" s="2">
         <v>1</v>
@@ -493,13 +499,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="B4" s="2">
-        <v>7.0000000000000001E-3</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="C4" s="2">
-        <v>7.0000000000000001E-3</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="D4" s="2">
         <v>1</v>
@@ -507,7 +513,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B5" s="2">
         <v>7.0000000000000001E-3</v>
@@ -521,7 +527,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B6" s="2">
         <v>7.0000000000000001E-3</v>
@@ -535,7 +541,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B7" s="2">
         <v>7.0000000000000001E-3</v>
@@ -549,7 +555,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B8" s="2">
         <v>7.0000000000000001E-3</v>
@@ -563,13 +569,13 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B9" s="2">
         <v>7.0000000000000001E-3</v>
       </c>
       <c r="C9" s="2">
-        <v>0.02</v>
+        <v>7.0000000000000001E-3</v>
       </c>
       <c r="D9" s="2">
         <v>1</v>
@@ -577,13 +583,13 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B10" s="2">
         <v>7.0000000000000001E-3</v>
       </c>
       <c r="C10" s="2">
-        <v>0.02</v>
+        <v>7.0000000000000001E-3</v>
       </c>
       <c r="D10" s="2">
         <v>1</v>
@@ -591,7 +597,7 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B11" s="2">
         <v>7.0000000000000001E-3</v>
@@ -605,7 +611,7 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B12" s="2">
         <v>7.0000000000000001E-3</v>
@@ -619,7 +625,7 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B13" s="2">
         <v>7.0000000000000001E-3</v>
@@ -633,7 +639,7 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B14" s="2">
         <v>7.0000000000000001E-3</v>
@@ -647,7 +653,7 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B15" s="2">
         <v>7.0000000000000001E-3</v>
@@ -661,7 +667,7 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B16" s="2">
         <v>7.0000000000000001E-3</v>
@@ -670,6 +676,34 @@
         <v>0.02</v>
       </c>
       <c r="D16" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="C17" s="2">
+        <v>0.02</v>
+      </c>
+      <c r="D17" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B18" s="2">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="C18" s="2">
+        <v>0.02</v>
+      </c>
+      <c r="D18" s="2">
         <v>1</v>
       </c>
     </row>

</xml_diff>